<commit_message>
Update PL28 Excel sequence to continue from 49
</commit_message>
<xml_diff>
--- a/Data Invoice/PL28_Packing_List.xlsx
+++ b/Data Invoice/PL28_Packing_List.xlsx
@@ -604,7 +604,7 @@
     </row>
     <row r="2" spans="1:13">
       <c r="A2">
-        <v>1</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
@@ -645,7 +645,7 @@
     </row>
     <row r="3" spans="1:13">
       <c r="A3">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -686,7 +686,7 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
@@ -727,7 +727,7 @@
     </row>
     <row r="5" spans="1:13">
       <c r="A5">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
@@ -768,7 +768,7 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
         <v>13</v>
@@ -809,7 +809,7 @@
     </row>
     <row r="7" spans="1:13">
       <c r="A7">
-        <v>6</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
         <v>13</v>
@@ -850,7 +850,7 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8">
-        <v>7</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
         <v>13</v>
@@ -891,7 +891,7 @@
     </row>
     <row r="9" spans="1:13">
       <c r="A9">
-        <v>8</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
@@ -932,7 +932,7 @@
     </row>
     <row r="10" spans="1:13">
       <c r="A10">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
         <v>13</v>
@@ -973,7 +973,7 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="B11" t="s">
         <v>13</v>
@@ -1014,7 +1014,7 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12">
-        <v>11</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
         <v>13</v>
@@ -1055,7 +1055,7 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="B13" t="s">
         <v>13</v>
@@ -1096,7 +1096,7 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="B14" t="s">
         <v>13</v>
@@ -1137,7 +1137,7 @@
     </row>
     <row r="15" spans="1:13">
       <c r="A15">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="B15" t="s">
         <v>13</v>
@@ -1178,7 +1178,7 @@
     </row>
     <row r="16" spans="1:13">
       <c r="A16">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="B16" t="s">
         <v>13</v>
@@ -1219,7 +1219,7 @@
     </row>
     <row r="17" spans="1:13">
       <c r="A17">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="B17" t="s">
         <v>13</v>
@@ -1260,7 +1260,7 @@
     </row>
     <row r="18" spans="1:13">
       <c r="A18">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="B18" t="s">
         <v>13</v>
@@ -1301,7 +1301,7 @@
     </row>
     <row r="19" spans="1:13">
       <c r="A19">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="B19" t="s">
         <v>13</v>
@@ -1342,7 +1342,7 @@
     </row>
     <row r="20" spans="1:13">
       <c r="A20">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="B20" t="s">
         <v>13</v>
@@ -1383,7 +1383,7 @@
     </row>
     <row r="21" spans="1:13">
       <c r="A21">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="B21" t="s">
         <v>13</v>
@@ -1424,7 +1424,7 @@
     </row>
     <row r="22" spans="1:13">
       <c r="A22">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="B22" t="s">
         <v>13</v>
@@ -1465,7 +1465,7 @@
     </row>
     <row r="23" spans="1:13">
       <c r="A23">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="B23" t="s">
         <v>13</v>
@@ -1506,7 +1506,7 @@
     </row>
     <row r="24" spans="1:13">
       <c r="A24">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="B24" t="s">
         <v>13</v>
@@ -1547,7 +1547,7 @@
     </row>
     <row r="25" spans="1:13">
       <c r="A25">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="B25" t="s">
         <v>13</v>
@@ -1588,7 +1588,7 @@
     </row>
     <row r="26" spans="1:13">
       <c r="A26">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="B26" t="s">
         <v>13</v>
@@ -1629,7 +1629,7 @@
     </row>
     <row r="27" spans="1:13">
       <c r="A27">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="B27" t="s">
         <v>13</v>
@@ -1670,7 +1670,7 @@
     </row>
     <row r="28" spans="1:13">
       <c r="A28">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="B28" t="s">
         <v>13</v>
@@ -1711,7 +1711,7 @@
     </row>
     <row r="29" spans="1:13">
       <c r="A29">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="B29" t="s">
         <v>13</v>
@@ -1752,7 +1752,7 @@
     </row>
     <row r="30" spans="1:13">
       <c r="A30">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="B30" t="s">
         <v>13</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="31" spans="1:13">
       <c r="A31">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="B31" t="s">
         <v>13</v>
@@ -1834,7 +1834,7 @@
     </row>
     <row r="32" spans="1:13">
       <c r="A32">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="B32" t="s">
         <v>13</v>
@@ -1875,7 +1875,7 @@
     </row>
     <row r="33" spans="1:13">
       <c r="A33">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="B33" t="s">
         <v>13</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="34" spans="1:13">
       <c r="A34">
-        <v>33</v>
+        <v>81</v>
       </c>
       <c r="B34" t="s">
         <v>13</v>
@@ -1957,7 +1957,7 @@
     </row>
     <row r="35" spans="1:13">
       <c r="A35">
-        <v>34</v>
+        <v>82</v>
       </c>
       <c r="B35" t="s">
         <v>13</v>
@@ -1998,7 +1998,7 @@
     </row>
     <row r="36" spans="1:13">
       <c r="A36">
-        <v>35</v>
+        <v>83</v>
       </c>
       <c r="B36" t="s">
         <v>13</v>
@@ -2039,7 +2039,7 @@
     </row>
     <row r="37" spans="1:13">
       <c r="A37">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="B37" t="s">
         <v>13</v>
@@ -2080,7 +2080,7 @@
     </row>
     <row r="38" spans="1:13">
       <c r="A38">
-        <v>37</v>
+        <v>85</v>
       </c>
       <c r="B38" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Allow no-space prefix for PL receiving and cutting
</commit_message>
<xml_diff>
--- a/Data Invoice/PL28_Packing_List.xlsx
+++ b/Data Invoice/PL28_Packing_List.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus 444\Desktop\Wood-Chatbot\whatsapp-bot\Data Invoice\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A3F4E9-2A45-413D-B4B5-DAEE8FE74DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -232,8 +238,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -266,17 +272,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -314,7 +328,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -348,6 +362,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -382,9 +397,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -557,11 +573,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M38"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -602,7 +618,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>49</v>
       </c>
@@ -643,7 +659,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>50</v>
       </c>
@@ -684,7 +700,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>51</v>
       </c>
@@ -725,7 +741,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>52</v>
       </c>
@@ -766,7 +782,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>53</v>
       </c>
@@ -807,7 +823,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>54</v>
       </c>
@@ -848,7 +864,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>55</v>
       </c>
@@ -889,7 +905,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>56</v>
       </c>
@@ -930,7 +946,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>57</v>
       </c>
@@ -971,7 +987,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>58</v>
       </c>
@@ -1012,7 +1028,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>59</v>
       </c>
@@ -1053,7 +1069,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>60</v>
       </c>
@@ -1094,7 +1110,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>61</v>
       </c>
@@ -1135,7 +1151,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>62</v>
       </c>
@@ -1176,7 +1192,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>63</v>
       </c>
@@ -1217,7 +1233,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>64</v>
       </c>
@@ -1258,7 +1274,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>65</v>
       </c>
@@ -1299,7 +1315,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>66</v>
       </c>
@@ -1340,7 +1356,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>67</v>
       </c>
@@ -1381,7 +1397,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>68</v>
       </c>
@@ -1422,7 +1438,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>69</v>
       </c>
@@ -1463,7 +1479,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>70</v>
       </c>
@@ -1489,7 +1505,7 @@
         <v>1320</v>
       </c>
       <c r="I23">
-        <v>1.144</v>
+        <v>1.1439999999999999</v>
       </c>
       <c r="J23">
         <v>0</v>
@@ -1504,7 +1520,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>71</v>
       </c>
@@ -1545,7 +1561,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>72</v>
       </c>
@@ -1586,7 +1602,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>73</v>
       </c>
@@ -1627,7 +1643,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>74</v>
       </c>
@@ -1668,7 +1684,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>75</v>
       </c>
@@ -1709,7 +1725,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>76</v>
       </c>
@@ -1750,7 +1766,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>77</v>
       </c>
@@ -1776,7 +1792,7 @@
         <v>1560</v>
       </c>
       <c r="I30">
-        <v>1.035</v>
+        <v>1.0349999999999999</v>
       </c>
       <c r="J30">
         <v>0</v>
@@ -1791,7 +1807,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>78</v>
       </c>
@@ -1817,7 +1833,7 @@
         <v>1560</v>
       </c>
       <c r="I31">
-        <v>1.035</v>
+        <v>1.0349999999999999</v>
       </c>
       <c r="J31">
         <v>0</v>
@@ -1832,7 +1848,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>79</v>
       </c>
@@ -1858,7 +1874,7 @@
         <v>1560</v>
       </c>
       <c r="I32">
-        <v>1.035</v>
+        <v>1.0349999999999999</v>
       </c>
       <c r="J32">
         <v>0</v>
@@ -1873,7 +1889,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>80</v>
       </c>
@@ -1899,7 +1915,7 @@
         <v>1560</v>
       </c>
       <c r="I33">
-        <v>1.035</v>
+        <v>1.0349999999999999</v>
       </c>
       <c r="J33">
         <v>0</v>
@@ -1914,7 +1930,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="34" spans="1:13">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>81</v>
       </c>
@@ -1940,7 +1956,7 @@
         <v>1644</v>
       </c>
       <c r="I34">
-        <v>1.134</v>
+        <v>1.1339999999999999</v>
       </c>
       <c r="J34">
         <v>0</v>
@@ -1955,7 +1971,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>82</v>
       </c>
@@ -1981,7 +1997,7 @@
         <v>1644</v>
       </c>
       <c r="I35">
-        <v>1.134</v>
+        <v>1.1339999999999999</v>
       </c>
       <c r="J35">
         <v>0</v>
@@ -1996,7 +2012,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="36" spans="1:13">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>83</v>
       </c>
@@ -2022,7 +2038,7 @@
         <v>1644</v>
       </c>
       <c r="I36">
-        <v>1.134</v>
+        <v>1.1339999999999999</v>
       </c>
       <c r="J36">
         <v>0</v>
@@ -2037,7 +2053,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>84</v>
       </c>
@@ -2063,7 +2079,7 @@
         <v>1644</v>
       </c>
       <c r="I37">
-        <v>1.134</v>
+        <v>1.1339999999999999</v>
       </c>
       <c r="J37">
         <v>0</v>
@@ -2078,7 +2094,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>85</v>
       </c>
@@ -2104,7 +2120,7 @@
         <v>1644</v>
       </c>
       <c r="I38">
-        <v>1.025</v>
+        <v>1.0249999999999999</v>
       </c>
       <c r="J38">
         <v>0</v>
@@ -2121,5 +2137,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>